<commit_message>
feat(gantry): migrate to EtherNet/IP motion and CellNetL2 real-time protocol
Squash merge of feat/EIP_Dev. Adds W5500 SPI driver, EtherNet/IP Class 1 originator stack for Kinetix/Rexroth drives, and CellNetL2 raw Ethernet framing. Removes deprecated MQTT, pulse-motor libraries, and legacy technical debt.
</commit_message>
<xml_diff>
--- a/driver_datasheets_and_calculations/WIRE_SIZE_SELECTION.xlsx
+++ b/driver_datasheets_and_calculations/WIRE_SIZE_SELECTION.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="X axis" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Z axis" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theta" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motion IO IF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EIP network" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gripper" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controller" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Still need to source" sheetId="11" state="visible" r:id="rId11"/>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'X axis'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Z axis'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Theta'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Motion IO IF'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'EIP network'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Gripper'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Controller'!$A$1:$O$1</definedName>
   </definedNames>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pneumatic (24 V valve from ESP32/MCP)</t>
+          <t>Pneumatic (24 V valve from ESP32 GPIO4)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PTI and digital I/O are signal cables (22-24 AWG STP); motion signals route WT32/MCP → Motion I/O IF (opto) → TBIO/HCS01.</t>
+          <t>Motion control is EtherNet/IP only — no PTI/opto production harness.</t>
         </is>
       </c>
     </row>
@@ -685,41 +685,53 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Logic-side IF harness (WT32/MCP → opto board) stays inside controller box; field-side IF → drive uses STP with FIELD_0V star.</t>
+          <t>Limit switches wire to drive TBIO / HCS01 X31 (NC sinking), not to the ESP32.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Key rule</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>See docs/HV_LV_SCHEMATICS.md and docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Order-provided cabling</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>See sheet 'Order-provided cabling' for McMc PO P0078269 and Youngblood OA 1693058 line items.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>On-hand inventory</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Wire: 16 / 18 AWG, 2-pair 22 AWG. Breakers: 1489-M2D010/020/100/400 — see inventory + panel breaker sheets.</t>
         </is>
@@ -847,17 +859,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 SPI</t>
+          <t>W5500 SPI (short harness)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>WT32-ETH01</t>
+          <t>WT32-ETH01 SPI pins</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17</t>
+          <t>W5500 Ethernet controller</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -885,7 +897,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>&lt;0.5 m</t>
+          <t>&lt;0.3 m</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -895,17 +907,17 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>SPI + reset/CS</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Direct MCP — not through Motion I/O IF. CS=15, MOSI=12, MISO=35, SCLK=5.</t>
+          <t>Keep SPI run short on controller PCB/harness. No Motion I/O IF / MCP production path.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>gantry_app_constants.h</t>
+          <t>docs/LOW_LEVEL_GANTRY_CONTROL.md</t>
         </is>
       </c>
     </row>
@@ -920,22 +932,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Logic harness to Motion I/O IF</t>
+          <t>EtherNet/IP originator link</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>WT32 GPIO14/2/0 + MCP23S17</t>
+          <t>W5500 RJ45</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF board (logic side)</t>
+          <t>X drive PORT1 (daisy-chain start)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>22 AWG (in-box)</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -954,11 +966,11 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>&lt;1 m total</t>
+          <t>As required</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -968,17 +980,17 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>3.3 V logic → 74AHCT244</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>One wire per motion signal to IF board. Keep short inside controller enclosure.</t>
+          <t>W5500 is EIP originator; X-&gt;Z-&gt;(Theta deferred) daisy-chain. Plant/MQTT may use WT32 RMII separately.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -993,27 +1005,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>5 V IF board supply</t>
+          <t>Gripper GPIO -&gt; relay</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>24 VDC panel bus</t>
+          <t>WT32-ETH01 GPIO4</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF 5 V regulator (PS-IF1)</t>
+          <t>CR1 coil (24 V relay)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18 AWG</t>
+          <t>22 AWG</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>LM2596 or 7805 module</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1041,17 +1053,17 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>~300 mA</t>
+          <t>3.3 V logic -&gt; relay coil driver</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Powers 74AHCT244 + opto LED side. LOGIC_GND only.</t>
+          <t>CR1 contacts feed 24 V to pneumatic valve. See Gripper sheet.</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>gantry_app_constants.h</t>
         </is>
       </c>
     </row>
@@ -1066,17 +1078,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Ethernet (optional)</t>
+          <t>Plant Ethernet (optional)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>WT32-ETH01</t>
+          <t>WT32-ETH01 RMII PHY</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plant network</t>
+          <t>Plant network / MQTT broker</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1119,12 +1131,12 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Standard patch cable — not on order.</t>
+          <t>Standard patch cable — not on order. Separate from W5500 EIP daisy-chain.</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>WT32_ETH01_PINOUT.md</t>
+          <t>pinout.csv / docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1186,12 +1198,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O opto interface (§9.1 BOM)</t>
+          <t>WIZ850io / W5500 module</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1 kit</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1201,7 +1213,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>HCPL-2530×3, VO14642AT×5, HCPL-3700×2, SN74AHCT244×2</t>
+          <t>WIZ850io</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1211,71 +1223,71 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>See docs/MOTION_IO_INTERFACE.md and generate_bom.py §9.1</t>
+          <t>EIP originator SPI Ethernet — see BOM §9.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>5 V regulator module (IF board)</t>
+          <t>Cat5e patch (EIP daisy-chain)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2–3</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>LM2596 or 7805</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Controller box</t>
+          <t>W5500↔X↔Z↔PC</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>24 V in → 5 V ~300 mA for AHCT + opto LEDs</t>
+          <t>Exclusive uplink with PC tools</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IF board terminal blocks</t>
+          <t>Limit switch STP to TBIO</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1 set</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>22 AWG STP</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Wago / Phoenix</t>
+          <t>Belden 8723</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Controller box</t>
+          <t>Actuator → TBIO</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Logic-side + field-side harness landing; FIELD_0V star</t>
+          <t>NC sinking; INPUT1-4 — not ESP32</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1607,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Breaker M2D010 on AC input to 24 V PSU</t>
+          <t>Use &gt;=2 A breaker (M2D010 undersized)</t>
         </is>
       </c>
     </row>
@@ -1691,19 +1703,19 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18–22 AWG spec — use inventory</t>
+          <t>GPIO4 → CR1 → valve</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG (signal harnesses)</t>
+          <t>2-pair 22 AWG (limits / SPI)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>~10–14</t>
+          <t>~4–6</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1723,103 +1735,39 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Logic IF harness + limits + SPI; encoders deferred</t>
+          <t>Drive limits + short W5500 SPI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>18 AWG (backup signals / limits)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>Pneumatic tube 6 mm</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>~3 m</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>18 AWG</t>
+          <t>6 mm OD</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>On-hand 18 AWG</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Various</t>
+          <t>Gripper</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>TBIO accepts 16–30 AWG; use if 22 AWG runs out</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Pneumatic tube 6 mm</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>~3 m</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>6 mm OD</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Gripper</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
           <t>Not wire — purchase if not using M3 plate bores</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>MCP SPI (4 wires)</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>On-hand</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>&lt;0.5 m</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>1× 2-pair cable: CS, MOSI, MISO, SCLK</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1938,12 +1886,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Accepts 16-30 AWG field wiring for PTI, DIR, SON, ALM, etc.</t>
+          <t>Accepts 16-30 AWG field wiring for limits / field I/O</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Field-wire Motion I/O IF → TBIO (not WT32 directly).</t>
+          <t>Field-wire NC limits -&gt; TBIO INPUT1/2. Motion via EIP - no PTI harness.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2116,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Field-wire Motion I/O IF → TBIO.</t>
+          <t>Field-wire NC limits -&gt; TBIO INPUT3/4. Motion via EIP - no PTI harness.</t>
         </is>
       </c>
     </row>
@@ -2376,60 +2324,44 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Motion I/O interface board (opto parts — BOM §9.1; docs/MOTION_IO_INTERFACE.md)</t>
+          <t>WIZ850io / W5500 module and short SPI harness (if not already installed)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Logic harness WT32/MCP → Motion I/O IF (inside controller box)</t>
+          <t>Cat5e EIP daisy-chain jumpers (W5500 → X → Z → PC)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Field harness Motion I/O IF → 2198-TBIO (×2) and HCS01 X31</t>
+          <t>Limit switch wiring from Beta actuators → TBIO INPUT1-4 (NC sinking)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Limit switch wiring from Beta actuators → MCP (direct, not via IF)</t>
+          <t>Gripper pneumatic hose (6 mm) and 24 V solenoid valve + GPIO4→CR1 wiring</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Buffered encoder A/B from Kinetix → ESP32 (deferred)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Gripper pneumatic hose (6 mm) and 24 V solenoid valve + wiring</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>WT32 ↔ MCP23S17 SPI harness</t>
+          <t>Qualified safety relay / STO design (see docs/HV_LV_SCHEMATICS.md review register)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A22:I22"/>
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A21:I21"/>
@@ -2445,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2747,12 +2679,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Logic harness WT32/MCP → Motion I/O IF</t>
+          <t>W5500 SPI harness (short)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Controller box internal</t>
+          <t>WT32 ↔ WIZ850io</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -2762,7 +2694,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>11 motion signals + 5 V feed. Short runs; not routed to TBIO directly.</t>
+          <t>MOSI12/MISO35/SCLK5/CS15/RST14. Keep &lt;0.5 m.</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2706,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Field harness Motion I/O IF → TBIO (×2) + HCS01 X31</t>
+          <t>Limit switches → drive TBIO</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>IF board → drives</t>
+          <t>Beta actuators → INPUT1-4</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2789,7 +2721,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP preferred for field legs; 18 AWG OK at TBIO (16–30 AWG).</t>
+          <t>NC sinking to drives; not ESP32. 22 AWG STP preferred.</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2733,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Limit switches → MCP</t>
+          <t>Gripper 24 V solenoid valve</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Beta actuators → MCP23S17</t>
+          <t>GPIO4 → CR1 → valve coil</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -2816,24 +2748,24 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Direct MCP — not through Motion I/O IF. Low-current dry contacts.</t>
+          <t>Within 18–22 AWG spec. Size fuse to coil nameplate.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>18 AWG</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Gripper 24 V solenoid valve</t>
+          <t>EIP daisy-chain</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Panel/MCP → valve coil</t>
+          <t>W5500 → X → Z → PC</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2843,7 +2775,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Within 18–22 AWG spec. Size fuse to coil nameplate.</t>
+          <t>Class 1 EtherNet/IP. Exclusive with PC prove tools.</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2787,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Logic side: X pulse + dir to IF (1 cable)</t>
+          <t>X limits MIN/MAX</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>GPIO14 + MCP DIR → Motion I/O IF</t>
+          <t>Beta 100-ZRS → TBIO INPUT1/2</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -2870,7 +2802,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Pair 1: pulse. Pair 2: dir. Stays in controller box.</t>
+          <t>Forward/Reverse Limit in KNX5100C.</t>
         </is>
       </c>
     </row>
@@ -2882,12 +2814,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Logic side: X SON + ARST to IF (1 cable)</t>
+          <t>Z limits MIN/MAX</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>MCP → Motion I/O IF</t>
+          <t>Beta 80-SRS → TBIO INPUT3/4</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -2897,7 +2829,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Pair 1: SON. Pair 2: ARST.</t>
+          <t>Forward/Reverse Limit in KNX5100C.</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2841,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Logic side: X ALM from IF (1 cable)</t>
+          <t>W5500 SPI (1 cable)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF → MCP A4</t>
+          <t>WT32 ↔ WIZ850io</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -2924,400 +2856,184 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>HCPL-3700 output back to MCP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Field side: IF → X TBIO (1–2 cables)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF → 2198-TBIO</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 1–2 cables</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Five motion signals + APWR/BPWR. Shield at drive end only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Logic side: Z pulse + dir to IF (1 cable)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>GPIO2 + MCP → Motion I/O IF</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 1 cable</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>GPIO2 is boot strap — keep LOW at reset.</t>
+          <t>4–5 wires short run. No MCP production path.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Logic + field: Z motion signals via IF</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF ↔ Z TBIO</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 2–3 cables</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Same pattern as X: logic in-box, field STP to TBIO.</t>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Quick summary</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>1489-M2D400</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>X limits MIN/MAX (1 cable)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Beta 100-ZRS → MCP</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 1 cable</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Direct MCP — not through IF board.</t>
+          <t>Assign to</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>X Kinetix E1020 AC input (via 2198-DB127-F line filter)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>1489-M2D100</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Z limits MIN/MAX (1 cable)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Beta 80-SRS → MCP</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 1 cable</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Direct MCP — not through IF board.</t>
+          <t>Assign to</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Z Kinetix E1004 AC input (via 2198-DB111-F line filter)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>1489-M2D020</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Theta logic to IF + field to X31</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>GPIO0 + MCP → IF → HCS01</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 2 cables</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>GPIO0 boot strap — must be HIGH at reset.</t>
+          <t>Assign to</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>HCS01 Theta drive AC input</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>1489-M2D010</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 SPI (1 cable)</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>WT32 ↔ MCP</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Yes — 1 cable</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>4 wires: CS=15, MOSI=12, MISO=35, SCLK=5. Short run (&lt;0.5 m).</t>
+          <t>Assign to</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>AC feed to 24 VDC control PSU (not DC load)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>16 AWG on hand</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Optional encoder A/B — X/Z (deferred)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>K5100 buffered out → ESP32</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>No — deferred</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>AXIS_*_ENCODER_FEEDBACK_ENABLED=0 until AM26LV32 Phase B.</t>
+          <t>Use for</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Z + Theta AC branches, 24 V PSU AC feed, optional 24 V DC runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>16 AWG on hand</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Do NOT use for</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>X 40 A AC branch (needs 8 AWG); motor U/V/W (use ordered 2090 cables)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>18 AWG on hand</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Use for</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>All TBIO I/O, limits, gripper valve, 24 V DC distribution from PSU</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Quick summary</t>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2-pair 22 AWG on hand</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Minimum count</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>~10 cables (encoders deferred)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>1489-M2D400</t>
+          <t>2-pair 22 AWG on hand</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Assign to</t>
+          <t>With encoders (future)</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>X Kinetix E1020 AC input (via 2198-DB127-F line filter)</t>
+          <t>~12 cables total</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>1489-M2D100</t>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Still must buy</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Assign to</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Z Kinetix E1004 AC input (via 2198-DB111-F line filter)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>1489-M2D020</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Assign to</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>HCS01 Theta drive AC input</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>1489-M2D010</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Assign to</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>AC feed to 24 VDC control PSU (not DC load)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>16 AWG on hand</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Use for</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Z + Theta AC branches, 24 V PSU AC feed, optional 24 V DC runs</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>16 AWG on hand</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Do NOT use for</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>X 40 A AC branch (needs 8 AWG); motor U/V/W (use ordered 2090 cables)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>18 AWG on hand</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Use for</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>All TBIO I/O, limits, gripper valve, 24 V DC distribution from PSU</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG on hand</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Minimum count</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>~10 cables (encoders deferred)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG on hand</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>With encoders (future)</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>~12 cables total</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Still must buy</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>8 AWG (+ ground) for X AC branch; 24 VDC PSU; Motion I/O opto parts (BOM §9.1); pneumatic hose if needed</t>
+          <t>8 AWG (+ ground) for X AC branch; 24 VDC PSU; W5500 if missing; Cat5e EIP jumpers; limit STP; pneumatic hose if needed</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4019,22 +3735,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PTI pulse train</t>
+          <t>EtherNet/IP (PORT1)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>WT32-ETH01 GPIO14 (LEDC) → Motion I/O IF</t>
+          <t>Upstream daisy-chain (W5500 or prior drive PORT2)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS AX+/AX- (2198-TBIO)</t>
+          <t>2198-E1020-ERS PORT1</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4067,17 +3783,17 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Low mA signal; HCPL-2530 U1-A</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Logic: GPIO14 → IF board. Field: IF → TBIO pins 43/41; APWR pin 39 ← +24 V. See docs/MOTION_IO_INTERFACE.md.</t>
+          <t>Motion command/feedback via assemblies 104/154. No PTI production wiring.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md; 2198-IN020</t>
+          <t>docs/LOW_LEVEL_GANTRY_CONTROL.md</t>
         </is>
       </c>
     </row>
@@ -4092,22 +3808,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>EtherNet/IP (PORT2)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_X_DIR → Motion I/O IF</t>
+          <t>2198-E1020-ERS PORT2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS BX+/BX- (TBIO)</t>
+          <t>Next hop (Z PORT1 or PC)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4140,17 +3856,17 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Digital I/O; HCPL-2530 U1-B</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>MCP Port A bit 0 → IF → TBIO pins 36/37; BPWR pin 35 ← +24 V.</t>
+          <t>Daisy-chain continue.</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -4165,22 +3881,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Servo ON / enable</t>
+          <t>Limit switches MIN/MAX</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_X_ENABLE → Motion I/O IF</t>
+          <t>Beta 100-ZRS NC limits</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS SON input (TBIO)</t>
+          <t>TBIO INPUT1 pin9 / INPUT2 pin10</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>22-24 AWG STP</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4199,7 +3915,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -4213,17 +3929,17 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Digital I/O; VO14642AT U4</t>
+          <t>24 V sinking NC</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>IF → TBIO INPUT (assign SON in KNX5100C) + DCOM.</t>
+          <t>Assign Forward/Reverse Limit in KNX5100C. Not wired to ESP32.</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -4238,27 +3954,27 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Alarm status</t>
+          <t>24 V control power</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS ALM output (TBIO) → Motion I/O IF</t>
+          <t>24 VDC supply</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_X_ALARM_STATUS</t>
+          <t>2198-E1020-ERS CP (+/-)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>16-24 AWG</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1606-XLxxx (typical)</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -4286,17 +4002,17 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Digital input to MCP; HCPL-3700 U9</t>
+          <t>~1.4 A @ 24 V per drive family</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Drive ALM → IF (3700) → MCP A4. Active LOW, MCP pull-up.</t>
+          <t>24 V PSU and wiring not on either order.</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>AB_Kinetix5100_user_manual.pdf</t>
         </is>
       </c>
     </row>
@@ -4311,37 +4027,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Alarm reset</t>
+          <t>Line filter</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_X_ALARM_RESET → Motion I/O IF</t>
+          <t>Panel / mains</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS ARST input (TBIO)</t>
+          <t>2198-E1020-ERS</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Per filter terminations</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>2198-DB127-F</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>McMc L4; PO P0078269</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -4349,7 +4065,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>As required</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -4359,17 +4075,17 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Digital output from MCP; VO14642AT U5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>IF → TBIO INPUT (assign ARST). Pulsed to clear alarm.</t>
+          <t>Filter hardware on order; panel wiring to filter is field-installed.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>McMc order acknowledgement.pdf</t>
         </is>
       </c>
     </row>
@@ -4384,37 +4100,37 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Encoder A/B (deferred)</t>
+          <t>I/O terminal block</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS AMOUT+/BMOUT+</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>WT32 GPIO4 / GPIO36 (PCNT)</t>
+          <t>2198-E1020-ERS I/O connector</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP</t>
+          <t>16-30 AWG at TBIO</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>2198-TBIO</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>McMc L2; PO P0078269</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
@@ -4422,7 +4138,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>As required</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -4432,307 +4148,15 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Buffered TTL-level outputs</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Deferred — AXIS_X_ENCODER_FEEDBACK_ENABLED=0 until AM26LV32 Phase B.</t>
+          <t>TBIO for limits / field I/O — not PTI production harness.</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>X axis</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Limit switches MIN/MAX</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Beta 100-ZRS limits</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>MCP23S17 PIN_X_LIMIT_MIN / MAX</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>22-24 AWG STP</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Signal only</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>Switches on actuator; direct MCP — not through Motion I/O IF.</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>gantry_app_constants.h</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>X axis</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>24 V control power</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>24 VDC supply</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>2198-E1020-ERS CP (+/-)</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>16-24 AWG</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>1606-XLxxx (typical)</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>~1.4 A @ 24 V per drive family</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>24 V PSU and wiring not on either order.</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>AB_Kinetix5100_user_manual.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>X axis</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Line filter</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Panel / mains</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>2198-E1020-ERS</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Per filter terminations</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2198-DB127-F</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>McMc L4; PO P0078269</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Filter hardware on order; panel wiring to filter is field-installed.</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>McMc order acknowledgement.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>X axis</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>I/O terminal block</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>2198-E1020-ERS I/O connector</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>16-30 AWG at TBIO</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>2198-TBIO</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>McMc L2; PO P0078269</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>TBIO provides screw terminals for PTI/I/O field wiring — not pre-made harness.</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>McMc order acknowledgement.pdf</t>
         </is>
@@ -4750,7 +4174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5150,22 +4574,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PTI pulse train</t>
+          <t>EtherNet/IP (PORT1)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>WT32-ETH01 GPIO2 (LEDC) → Motion I/O IF</t>
+          <t>Upstream daisy-chain (X PORT2 or W5500)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS AX+/AX- (2198-TBIO)</t>
+          <t>2198-E1004-ERS PORT1</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5198,17 +4622,17 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>HCPL-2530 U2-A; GPIO2 boot strap</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Logic: GPIO2 → IF. Field: IF → Z TBIO APWR/AX±. Keep GPIO2 LOW at reset.</t>
+          <t>Motion command/feedback via assemblies 104/154. No PTI production wiring.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/LOW_LEVEL_GANTRY_CONTROL.md</t>
         </is>
       </c>
     </row>
@@ -5223,22 +4647,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>EtherNet/IP (PORT2)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_Z_DIR → Motion I/O IF</t>
+          <t>2198-E1004-ERS PORT2</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS BX+/BX- (TBIO)</t>
+          <t>Next hop (Theta PORT1 or PC)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5271,17 +4695,17 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>HCPL-2530 U2-B</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>MCP Port B bit 0 → IF → Z TBIO BPWR/BX±.</t>
+          <t>Daisy-chain continue.</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -5296,22 +4720,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Servo ON / enable</t>
+          <t>Limit switches MIN/MAX</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_Z_ENABLE → Motion I/O IF</t>
+          <t>Beta 80-SRS NC limits</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS SON input (TBIO)</t>
+          <t>TBIO INPUT3 pin11 / INPUT4 pin12</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>22-24 AWG STP</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5330,7 +4754,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -5344,17 +4768,17 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>VO14642AT U6</t>
+          <t>24 V sinking NC</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>IF → Z TBIO SON + DCOM.</t>
+          <t>Assign Forward/Reverse Limit in KNX5100C. Not wired to ESP32.</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -5369,27 +4793,27 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Alarm status</t>
+          <t>24 V control power</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS ALM output (TBIO) → Motion I/O IF</t>
+          <t>24 VDC supply</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_Z_ALARM_STATUS</t>
+          <t>2198-E1004-ERS CP (+/-)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>16-24 AWG</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1606-XLxxx (typical)</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -5417,17 +4841,17 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>HCPL-3700 U10</t>
+          <t>~1.4 A @ 24 V per drive family</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Drive ALM → IF → MCP B12.</t>
+          <t>24 V PSU and wiring not on either order.</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>AB_Kinetix5100_user_manual.pdf</t>
         </is>
       </c>
     </row>
@@ -5442,37 +4866,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Alarm reset</t>
+          <t>Line filter</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_Z_ALARM_RESET → Motion I/O IF</t>
+          <t>Panel / mains</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS ARST input (TBIO)</t>
+          <t>2198-E1004-ERS</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Per filter terminations</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>2198-DB111-F</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>McMc L16; PO P0078269</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -5480,7 +4904,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>As required</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -5490,17 +4914,17 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>VO14642AT U7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>MCP B13 → IF → Z TBIO ARST.</t>
+          <t>Filter hardware on order; panel wiring field-installed.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>McMc order acknowledgement.pdf</t>
         </is>
       </c>
     </row>
@@ -5515,45 +4939,45 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Encoder A/B (deferred)</t>
+          <t>I/O terminal block</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS buffered out</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>WT32 GPIO39 / GPIO32</t>
+          <t>2198-E1004-ERS I/O connector</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP</t>
+          <t>16-30 AWG at TBIO</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>2198-TBIO</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>McMc L12; PO P0078269</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>As required</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -5563,234 +4987,15 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>PCNT feedback</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Field-build harness. Phase B deferred — AXIS_Z_ENCODER_FEEDBACK_ENABLED=0.</t>
+          <t>TBIO for limits / field I/O — not PTI production harness.</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>PROGRAMMING_REFERENCE.md §12</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Z axis</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Limit switches MIN/MAX</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Beta 80-SRS limits</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>MCP23S17 PIN_Z_LIMIT_MIN / MAX</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>22-24 AWG STP</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>Direct MCP — not through Motion I/O IF. Field-installed.</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>gantry_app_constants.h</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Z axis</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>I/O terminal block</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>2198-E1004-ERS I/O connector</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>16-30 AWG at TBIO</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>2198-TBIO</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>McMc L12; PO P0078269</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>TBIO on order for Z drive.</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>McMc order acknowledgement.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Z axis</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Line filter</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Panel / mains</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>2198-E1004-ERS</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Per filter terminations</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>2198-DB111-F</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>McMc L16; PO P0078269</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Filter hardware on order; panel wiring field-installed.</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>McMc order acknowledgement.pdf</t>
         </is>
@@ -5808,7 +5013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6208,22 +5413,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Step pulse</t>
+          <t>EtherNet/IP (deferred)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>WT32-ETH01 GPIO0 → Motion I/O IF</t>
+          <t>Upstream daisy-chain (Z PORT2)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>HCS01 X31 step (pin TBD)</t>
+          <t>HCS01.1E multi-Ethernet PORT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -6256,17 +5461,17 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>HCPL-2530 U3-A</t>
+          <t>Class 1 EIP (future)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>GPIO0 boot strap — must be HIGH at reset. X31 pin map pending MPB doc.</t>
+          <t>Theta EIP originator path deferred — factory SCHUNK power/encoder cables only for now. No PTI/step-dir production wiring.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/LOW_LEVEL_GANTRY_CONTROL.md</t>
         </is>
       </c>
     </row>
@@ -6281,22 +5486,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>Limit switches (optional)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_THETA_DIR → Motion I/O IF</t>
+          <t>ERD / axis NC limits</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>HCS01 X31 dir (pin TBD)</t>
+          <t>HCS01 X31.5 / X31.6 digital inputs</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
+          <t>22-24 AWG STP</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6315,7 +5520,7 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -6329,90 +5534,17 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>HCPL-2530 U3-B</t>
+          <t>24 V sinking NC</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>MCP B14 → IF → HCS01 X31.</t>
+          <t>Optional drive-side limits on X31. Not wired to ESP32. Confirm X31 pin map in IndraDrive doc.</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Theta</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Drive enable</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>MCP23S17 PIN_THETA_ENABLE → Motion I/O IF</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>HCS01 X31 enable (pin TBD)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>22-24 AWG STP (field); 22 AWG logic</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>VO14642AT U8</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>MCP B15 → IF → HCS01 X31. FIELD_0V star at X31.9.</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -6428,7 +5560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6531,27 +5663,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF</t>
+          <t>EIP network</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Field harness to X TBIO</t>
+          <t>Cat5e daisy-chain</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF (field side)</t>
+          <t>W5500 -&gt; X PORT1 -&gt; X PORT2 -&gt; Z PORT1 -&gt; Z PORT2</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2198-E1020-ERS 2198-TBIO</t>
+          <t>(Theta EIP deferred)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>22-24 AWG STP</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -6570,7 +5702,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -6584,17 +5716,17 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>5 motion signals + APWR/BPWR</t>
+          <t>Class 1 EIP</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Pulse, dir, SON, ARST out; ALM in. Shield tied at drive end only.</t>
+          <t>No opto / PTI / MCP Motion I/O IF harness. Motion via EIP assemblies only.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -6604,22 +5736,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF</t>
+          <t>EIP network</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Field harness to Z TBIO</t>
+          <t>Limit STP to drives</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Motion I/O IF (field side)</t>
+          <t>Beta / ERD NC limits</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2198-E1004-ERS 2198-TBIO</t>
+          <t>X TBIO INPUT1/2; Z TBIO INPUT3/4; Theta X31.5/6 optional</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -6657,163 +5789,17 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Same pin map as X TBIO</t>
+          <t>24 V sinking NC</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Five motion signals + APWR/BPWR + DCOM to FIELD_0V star.</t>
+          <t>Shield at drive end only. Limits are drive-side — not ESP32 GPIO.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Field harness to HCS01 X31</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF (field side)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>HCS01.1E X31 Step/Dir</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>22-24 AWG STP</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Step, dir, enable</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>X31 pin numbers TBD. Tie X31.9 (0 V) to FIELD_0V star.</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>FIELD_0V + 24 V distribution</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>24 VDC PSU + K5100 DCOM</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Motion I/O IF terminal block</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>As required</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Star ground</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Single FIELD_0V star for both TBIO DCOM and HCS01 X31.9. Isolated from LOGIC_GND.</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>docs/MOTION_IO_INTERFACE.md</t>
+          <t>docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
     </row>
@@ -7015,12 +6001,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>24 VDC valve output</t>
+          <t>ESP32 GPIO4 -&gt; CR1 (24 V relay) -&gt; valve coil</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>MCP23S17 PIN_GRIPPER (Port A bit 7)</t>
+          <t>24 VDC pneumatic solenoid</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -7063,7 +6049,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Valve and wiring not on either order.</t>
+          <t>GPIO4 drives CR1 coil side; CR1 contacts switch 24 V to valve. Not MCP23S17. Valve/relay not on either order.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">

</xml_diff>